<commit_message>
project and order files mangaed
</commit_message>
<xml_diff>
--- a/uploads/projects/fragrances_2025-04-28.xlsx
+++ b/uploads/projects/fragrances_2025-04-28.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Fragrances" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -398,10 +398,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K12"/>
+  <cols>
+    <col min="1" max="1" width="41.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" customWidth="1"/>
+    <col min="5" max="5" width="50.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="50.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>name</v>
+        <v>Name</v>
       </c>
       <c r="B1" t="str">
         <v>Brand</v>

</xml_diff>